<commit_message>
feat(ops): self-healing, remote health/update, session-race fix
Make the Pi appliance survivable unattended and safely self-updating,
and fix two issues found in a no-hardware real-click walkthrough.

- Sync never crashes the kiosk; systemd retries forever; GET /api/health
  + /dashboard give a non-Linux operator a browser liveness view.
- deploy/install/update.sh applies a release tarball from the M: share
  (stage->backup->swap->migrate->health-gate->auto-rollback); admin
  "Software Update" button + locked-down sudoers + transient systemd-run.
- Admin panel establishes its backend session on open (was 401-ing).
- get_session_factory returns a plain sessionmaker with per-session
  close; scoped_session.remove() under FastAPI's reused threadpool could
  close another request's session mid-commit (intermittent 500).
</commit_message>
<xml_diff>
--- a/sim/data/Messmittelliste.sample.xlsx
+++ b/sim/data/Messmittelliste.sample.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -502,7 +502,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>SN-FL-001</t>
+          <t>SN-FL-87V-01</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Scopemeter</t>
+          <t>Digital-Multimeter</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -534,12 +534,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ScopeMeter 120B</t>
+          <t>87V</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>SN-FL-002</t>
+          <t>SN-FL-87V-02</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -556,7 +556,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Kabeltester</t>
+          <t>Industrie-Multimeter</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -571,12 +571,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>MicroScanner2</t>
+          <t>287</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>SN-FL-003</t>
+          <t>SN-FL-287</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -588,91 +588,91 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1006</t>
+          <t>1004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Temperaturdatenlogger</t>
+          <t>Zangenmessgerät</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Schrank A6</t>
+          <t>Schrank A4</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Testo</t>
+          <t>Fluke</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>175T1</t>
+          <t>376 FC</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SN-TE-006</t>
+          <t>SN-FL-376</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Schrank A6</t>
+          <t>Schrank A4</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1004</t>
+          <t>1005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Zangenamperemeter</t>
+          <t>Temperaturdatenlogger</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Schrank A4</t>
+          <t>Schrank A5</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Fluke</t>
+          <t>Testo</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>376 FC</t>
+          <t>175T1</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>SN-FL-004</t>
+          <t>SN-TE-175</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Max Mustermann</t>
+          <t>Schrank A5</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1005</t>
+          <t>1006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Isolationsprüfer</t>
+          <t>Kabeltester</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Schrank A5</t>
+          <t>Schrank A6</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -682,17 +682,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1587 FC</t>
+          <t>MicroScanner2</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>SN-FL-005</t>
+          <t>SN-FL-MS2</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Anna Schmidt</t>
+          <t>Schrank A6</t>
         </is>
       </c>
     </row>
@@ -704,32 +704,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Drehmomentschlüssel</t>
+          <t>ScopeMeter</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Regal B1</t>
+          <t>Schrank A7</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Gedore</t>
+          <t>Fluke</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2642-05</t>
+          <t>ScopeMeter 120B</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>SN-GE-007</t>
+          <t>SN-FL-120</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Regal B1</t>
+          <t>Schrank A7</t>
         </is>
       </c>
     </row>
@@ -741,26 +741,135 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>Isolationsprüfer</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Schrank A8</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Fluke</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1587 FC</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>SN-FL-1587</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Max Mustermann</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Leistungsmessgerät</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Schrank A9</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Fluke</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1736</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>SN-FL-1736</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Schrank A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Drehmomentschlüssel</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Regal B1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Gedore</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2642-05</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>SN-GE-2642</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Lukas Weber</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2002</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>Etikettendrucker</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Brady</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>M611</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>SN-BR-008</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>SN-BR-611</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>